<commit_message>
updated readme and included neighbour accuracy in test file
</commit_message>
<xml_diff>
--- a/Tests/Trilateration, fingerprint and fusion tests.xlsx
+++ b/Tests/Trilateration, fingerprint and fusion tests.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joryl\Dissertation\dissertation_project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joryl\Dissertation\dissertation_project\Tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A518341E-2B70-4D18-A5E3-F68C5412C161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{861249E9-DA27-46ED-AD9F-F80BFC4BB6FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{AEB7D5E0-1957-4899-B8BC-4609C2B69C7B}"/>
+    <workbookView xWindow="11328" yWindow="0" windowWidth="11712" windowHeight="12240" firstSheet="1" activeTab="1" xr2:uid="{AEB7D5E0-1957-4899-B8BC-4609C2B69C7B}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5858" uniqueCount="3011">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5861" uniqueCount="3012">
   <si>
     <t>cell 1</t>
   </si>
@@ -9075,6 +9075,9 @@
   </si>
   <si>
     <t>Incorrect cell</t>
+  </si>
+  <si>
+    <t>Including Neighbours Accuracy:</t>
   </si>
 </sst>
 </file>
@@ -24696,12 +24699,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76339025-29A5-4D55-8076-CA1CFDF72B94}">
-  <dimension ref="A1:T35"/>
+  <dimension ref="A1:T36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.88671875" customWidth="1"/>
     <col min="2" max="18" width="17.6640625" customWidth="1"/>
-    <col min="19" max="19" width="15.44140625" customWidth="1"/>
+    <col min="19" max="19" width="26.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
@@ -26426,6 +26429,14 @@
       </c>
       <c r="T35" s="3">
         <v>0.6</v>
+      </c>
+    </row>
+    <row r="36" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="S36" t="s">
+        <v>3011</v>
+      </c>
+      <c r="T36" s="3">
+        <v>0.98</v>
       </c>
     </row>
   </sheetData>
@@ -26441,7 +26452,8 @@
   <cols>
     <col min="1" max="1" width="13.109375" customWidth="1"/>
     <col min="2" max="2" width="27.109375" customWidth="1"/>
-    <col min="3" max="19" width="18.44140625" customWidth="1"/>
+    <col min="3" max="18" width="18.44140625" customWidth="1"/>
+    <col min="19" max="19" width="27.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
@@ -28166,6 +28178,14 @@
       </c>
       <c r="T36" s="3">
         <v>0.6</v>
+      </c>
+    </row>
+    <row r="37" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="S37" t="s">
+        <v>3011</v>
+      </c>
+      <c r="T37" s="3">
+        <v>0.95</v>
       </c>
     </row>
     <row r="229" spans="15:18" x14ac:dyDescent="0.3">
@@ -28191,13 +28211,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF6243FF-C0B6-418B-8085-027B7EE2F8DC}">
-  <dimension ref="A2:U36"/>
+  <dimension ref="A2:U37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="11.5546875" customWidth="1"/>
     <col min="3" max="3" width="8.88671875" customWidth="1"/>
-    <col min="20" max="20" width="13.44140625" customWidth="1"/>
+    <col min="20" max="20" width="27" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
@@ -29924,6 +29944,14 @@
         <v>0.7</v>
       </c>
     </row>
+    <row r="37" spans="2:21" x14ac:dyDescent="0.3">
+      <c r="T37" t="s">
+        <v>3011</v>
+      </c>
+      <c r="U37" s="3">
+        <v>0.97</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>